<commit_message>
Rename output_name/output_title fields, add language-specific titles and language param to run_outputs
Agent-Logs-Url: https://github.com/SaeedR1987/public_health_resources/sessions/2be185e7-4ed3-45cb-a75f-a2192328ee51

Co-authored-by: SaeedR1987 <17695865+SaeedR1987@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/resources/outputs_schema_data_analytics_demographics_template.xlsx
+++ b/resources/outputs_schema_data_analytics_demographics_template.xlsx
@@ -413,20 +413,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>output_title</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>output_name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>output_title</t>
-        </is>
-      </c>
       <c r="C1" t="inlineStr">
         <is>
           <t>output_subtitle</t>
@@ -470,6 +470,21 @@
       <c r="K1" t="inlineStr">
         <is>
           <t>dataset_type</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>output_title_english</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>output_title_french</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>output_title_arabic</t>
         </is>
       </c>
     </row>

</xml_diff>